<commit_message>
Enviada la version 2.1.1
</commit_message>
<xml_diff>
--- a/output/Datos Afip/Mis Comprobantes Emitidos - CUIT 20163254159 (1).xlsx
+++ b/output/Datos Afip/Mis Comprobantes Emitidos - CUIT 20163254159 (1).xlsx
@@ -381,7 +381,7 @@
     <row r="3">
       <c t="inlineStr" r="A3">
         <is>
-          <t>08/09/2025</t>
+          <t>06/10/2025</t>
         </is>
       </c>
       <c t="inlineStr" r="B3">
@@ -393,13 +393,13 @@
         <v>6</v>
       </c>
       <c r="D3" s="65">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E3" s="65">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F3" s="65">
-        <v>75369316553646</v>
+        <v>75409856217031</v>
       </c>
       <c t="inlineStr" r="G3">
         <is>
@@ -423,13 +423,13 @@
         </is>
       </c>
       <c r="S3" s="65">
-        <v>2100000</v>
+        <v>210000</v>
       </c>
       <c r="T3" s="65">
-        <v>10000000</v>
+        <v>1000000</v>
       </c>
       <c r="W3" s="65">
-        <v>10000000</v>
+        <v>1000000</v>
       </c>
       <c r="X3" s="65">
         <v>0</v>
@@ -441,10 +441,10 @@
         <v>0</v>
       </c>
       <c r="AA3" s="65">
-        <v>2100000</v>
+        <v>210000</v>
       </c>
       <c r="AB3" s="65">
-        <v>12100000</v>
+        <v>1210000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>